<commit_message>
feat: implement full-stack patient appointment management system with RPA automation workflows
</commit_message>
<xml_diff>
--- a/Data/Demandes_Patients.xlsx
+++ b/Data/Demandes_Patients.xlsx
@@ -1,17 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
-  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
-  <x:workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="164011"/>
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:workbookPr filterPrivacy="true" codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11820" firstSheet="0" activeTab="0"/>
+    <x:workbookView firstSheet="0" activeTab="0"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Demandes" sheetId="1" r:id="rId1"/>
   </x:sheets>
   <x:definedNames/>
-  <x:calcPr calcId="162913"/>
+  <x:calcPr calcId="125725"/>
 </x:workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35,6 +56,12 @@
     <x:t>Motif</x:t>
   </x:si>
   <x:si>
+    <x:t>DateRDV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HeureRDV</x:t>
+  </x:si>
+  <x:si>
     <x:t>Statut</x:t>
   </x:si>
   <x:si>
@@ -47,7 +74,7 @@
     <x:t>RDV-001</x:t>
   </x:si>
   <x:si>
-    <x:t>habib razeg</x:t>
+    <x:t>Laith Mahdi</x:t>
   </x:si>
   <x:si>
     <x:t>+21653843799</x:t>
@@ -59,28 +86,46 @@
     <x:t>Masculin</x:t>
   </x:si>
   <x:si>
+    <x:t>Consultation générale</x:t>
+  </x:si>
+  <x:si>
+    <x:t>27/04/2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>09:30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Traité</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>RDV-002</x:t>
+  </x:si>
+  <x:si>
+    <x:t>dalel loussief</x:t>
+  </x:si>
+  <x:si>
+    <x:t>mahdi.laith@itbs.tn</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Féminin</x:t>
+  </x:si>
+  <x:si>
     <x:t>Renouvellement ordonnance</x:t>
-  </x:si>
-  <x:si>
-    <x:t>27/04/2026</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>Traité</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac x16r2">
+<x:styleSheet xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
+    <x:numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
   </x:numFmts>
-  <x:fonts count="2" x14ac:knownFonts="1">
+  <x:fonts count="2">
     <x:font>
-      <x:sz val="11"/>
+      <x:sz val="12"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
       <x:family val="2"/>
@@ -115,20 +160,12 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
   <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
   </x:cellStyles>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </x:ext>
-    <x:ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </x:ext>
-  </x:extLst>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </x:styleSheet>
 </file>
 
@@ -143,44 +180,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -210,12 +247,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -254,164 +291,223 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:I2"/>
-  <x:sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <x:dimension ref="A1:K3"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="15" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" style="0" customWidth="1"/>
-    <x:col min="7" max="8" width="15" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="40" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10.832031" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25.832031" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.832031" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25.832031" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.832031" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25.832031" style="0" customWidth="1"/>
+    <x:col min="7" max="9" width="15.832031" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="40.832031" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <x:row r="1" spans="1:11">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
@@ -439,41 +535,91 @@
       <x:c r="I1" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
+      <x:c r="J1" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K1" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
-    <x:row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <x:row r="2" spans="1:11">
       <x:c r="A2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
         <x:v>17</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:11">
+      <x:c r="A3" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>20</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="portrait" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
+  <x:ignoredErrors>
+    <x:ignoredError sqref="A1:K3" numberStoredAsText="1"/>
+  </x:ignoredErrors>
   <x:tableParts count="0"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement agenda availability checking logic and add required workflow files and data sources
</commit_message>
<xml_diff>
--- a/Data/Demandes_Patients.xlsx
+++ b/Data/Demandes_Patients.xlsx
@@ -38,6 +38,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
+    <x:t>Notes</x:t>
+  </x:si>
+  <x:si>
     <x:t>ID</x:t>
   </x:si>
   <x:si>
@@ -68,19 +71,19 @@
     <x:t>DateDemande</x:t>
   </x:si>
   <x:si>
-    <x:t>Notes</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RDV-001</x:t>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>RDV-003</x:t>
   </x:si>
   <x:si>
     <x:t>Laith Mahdi</x:t>
   </x:si>
   <x:si>
-    <x:t>+21653843799</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mahdilaith08@gmail.com</x:t>
+    <x:t>53843799</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mahdilaith08@gmail.com</x:t>
   </x:si>
   <x:si>
     <x:t>Masculin</x:t>
@@ -98,19 +101,16 @@
     <x:t>Traité</x:t>
   </x:si>
   <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>RDV-002</x:t>
-  </x:si>
-  <x:si>
-    <x:t>dalel loussief</x:t>
+    <x:t>RDV-004</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Yassine mahdi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>+216 53 843 799</x:t>
   </x:si>
   <x:si>
     <x:t>mahdi.laith@itbs.tn</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Féminin</x:t>
   </x:si>
   <x:si>
     <x:t>Renouvellement ordonnance</x:t>
@@ -494,7 +494,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K3"/>
+  <x:dimension ref="A1:K5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10.832031" style="0" customWidth="1"/>
@@ -547,69 +547,139 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="K2" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:11">
       <x:c r="A3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11">
+      <x:c r="A4" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11">
+      <x:c r="A5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
+      <x:c r="C5" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
+      <x:c r="D5" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="E3" s="0" t="s">
+      <x:c r="E5" s="0" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="F3" s="0" t="s">
+      <x:c r="F5" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
+      <x:c r="H5" s="0" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I3" s="0" t="s">
+      <x:c r="I5" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="J3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K3" s="0" t="s">
+      <x:c r="J5" s="0" t="s">
         <x:v>20</x:v>
+      </x:c>
+      <x:c r="K5" s="0" t="s">
+        <x:v>18</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -618,7 +688,7 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:ignoredErrors>
-    <x:ignoredError sqref="A1:K3" numberStoredAsText="1"/>
+    <x:ignoredError sqref="A1:K5" numberStoredAsText="1"/>
   </x:ignoredErrors>
   <x:tableParts count="0"/>
 </x:worksheet>

</xml_diff>